<commit_message>
graphe JS : colonne txn_dta (transformation) + tableaux successeurs/predecesseurs
Ajoute la colonne txn_dta en fin de fichier Excel : la transformation portee
par chaque arete. Le panneau du noeud selectionne affiche desormais deux
tableaux (successeur/transformation, predecesseur/transformation) a la place
des puces simples.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/javascript/exemple.xlsx
+++ b/javascript/exemple.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:J21"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -427,6 +427,9 @@
       <c r="I1" t="str">
         <v>edg_4</v>
       </c>
+      <c r="J1" t="str">
+        <v>txn_dta</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -456,6 +459,9 @@
       <c r="I2" t="str">
         <v>EA4</v>
       </c>
+      <c r="J2" t="str">
+        <v>agrégation</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -485,6 +491,9 @@
       <c r="I3" t="str">
         <v>EA4</v>
       </c>
+      <c r="J3" t="str">
+        <v>filtre</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -514,6 +523,9 @@
       <c r="I4" t="str">
         <v>EA4</v>
       </c>
+      <c r="J4" t="str">
+        <v>jointure</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -543,6 +555,9 @@
       <c r="I5" t="str">
         <v>EB4</v>
       </c>
+      <c r="J5" t="str">
+        <v>tri</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -572,6 +587,9 @@
       <c r="I6" t="str">
         <v>EB4</v>
       </c>
+      <c r="J6" t="str">
+        <v>calcul</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -601,6 +619,9 @@
       <c r="I7" t="str">
         <v>EB4</v>
       </c>
+      <c r="J7" t="str">
+        <v>arrondi</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -630,6 +651,9 @@
       <c r="I8" t="str">
         <v>EC4</v>
       </c>
+      <c r="J8" t="str">
+        <v>normalisation</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
@@ -659,6 +683,9 @@
       <c r="I9" t="str">
         <v>EC4</v>
       </c>
+      <c r="J9" t="str">
+        <v>concaténation</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
@@ -688,6 +715,9 @@
       <c r="I10" t="str">
         <v>ED4</v>
       </c>
+      <c r="J10" t="str">
+        <v>déduplication</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
@@ -717,6 +747,9 @@
       <c r="I11" t="str">
         <v>ED4</v>
       </c>
+      <c r="J11" t="str">
+        <v>conversion</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
@@ -746,6 +779,9 @@
       <c r="I12" t="str">
         <v>EE4</v>
       </c>
+      <c r="J12" t="str">
+        <v>filtre</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
@@ -775,6 +811,9 @@
       <c r="I13" t="str">
         <v>EE4</v>
       </c>
+      <c r="J13" t="str">
+        <v>agrégation</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
@@ -804,6 +843,9 @@
       <c r="I14" t="str">
         <v>EF4</v>
       </c>
+      <c r="J14" t="str">
+        <v>jointure</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
@@ -833,6 +875,9 @@
       <c r="I15" t="str">
         <v>EF4</v>
       </c>
+      <c r="J15" t="str">
+        <v>tri</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
@@ -862,6 +907,9 @@
       <c r="I16" t="str">
         <v>EF4</v>
       </c>
+      <c r="J16" t="str">
+        <v>calcul</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
@@ -891,6 +939,9 @@
       <c r="I17" t="str">
         <v>EC4</v>
       </c>
+      <c r="J17" t="str">
+        <v>arrondi</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
@@ -920,6 +971,9 @@
       <c r="I18" t="str">
         <v>EE4</v>
       </c>
+      <c r="J18" t="str">
+        <v>normalisation</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
@@ -949,6 +1003,9 @@
       <c r="I19" t="str">
         <v>EA4</v>
       </c>
+      <c r="J19" t="str">
+        <v>concaténation</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
@@ -978,6 +1035,9 @@
       <c r="I20" t="str">
         <v>EB4</v>
       </c>
+      <c r="J20" t="str">
+        <v>déduplication</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
@@ -1007,10 +1067,13 @@
       <c r="I21" t="str">
         <v>EA4</v>
       </c>
+      <c r="J21" t="str">
+        <v>conversion</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J21"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>